<commit_message>
Added sonar qube analysis.
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Laptop\e\VVSS\CamiVVSS_ro2025-2026\Labs\CheckListsAll\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{EFE83867-3721-469D-B0A3-67FDA22FF09F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D56FFB0-A547-4ED8-AC29-34132A9A46AE}"/>
+  <xr:revisionPtr revIDLastSave="122" documentId="13_ncr:1_{EFE83867-3721-469D-B0A3-67FDA22FF09F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DAD67BE2-A3EB-49C8-95C1-F2675151D60C}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="650" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="95">
   <si>
     <t>do not print this form</t>
   </si>
@@ -71,6 +71,9 @@
     <t>Student 2:</t>
   </si>
   <si>
+    <t>Vitelaru Teodor</t>
+  </si>
+  <si>
     <t>Author Name:</t>
   </si>
   <si>
@@ -80,10 +83,16 @@
     <t>Student 3:</t>
   </si>
   <si>
+    <t>Ursoiu Calin</t>
+  </si>
+  <si>
     <t>Reviewer Name:</t>
   </si>
   <si>
     <t xml:space="preserve">Review date: </t>
+  </si>
+  <si>
+    <t>14/03/2026</t>
   </si>
   <si>
     <t>Crt. No.</t>
@@ -295,6 +304,9 @@
     <t>Tool used:</t>
   </si>
   <si>
+    <t>SonarQube</t>
+  </si>
+  <si>
     <t>File, Line</t>
   </si>
   <si>
@@ -307,7 +319,72 @@
     <t>After/Argument</t>
   </si>
   <si>
-    <t>Effort to perform tool-based code analysis (hours):</t>
+    <t>AbstractRepository.java:37</t>
+  </si>
+  <si>
+    <t>Metoda de save e identica cu cea de update.</t>
+  </si>
+  <si>
+    <t>AbstractRepository.java:20</t>
+  </si>
+  <si>
+    <t>Un cast redundant.</t>
+  </si>
+  <si>
+    <t>return (List&lt;E&gt;)StreamSupport.stream(entities.values().spliterator(), false).toList();
+//                    .collect(Collectors.toList());</t>
+  </si>
+  <si>
+    <t>return StreamSupport.stream(entities.values().spliterator(),</t>
+  </si>
+  <si>
+    <t>DailyReportService.java:21</t>
+  </si>
+  <si>
+    <t>Instructiuni comentate si nefolosite,</t>
+  </si>
+  <si>
+    <t>List&lt;Order&gt; orders = StreamSupport.stream(repo.findAll().spliterator(), false)
+//                .collect(Collectors.toList());
+        return repo.findAll().size();</t>
+  </si>
+  <si>
+    <t>public int getTotalOrders() {
+        return repo.findAll().size();
+    }</t>
+  </si>
+  <si>
+    <t>DailyReportService.java:6</t>
+  </si>
+  <si>
+    <t>Importuri nefolosite</t>
+  </si>
+  <si>
+    <t>import java.util.List;
+import java.util.stream.Collectors;
+import java.util.stream.StreamSupport;</t>
+  </si>
+  <si>
+    <t>ProductService.java:31</t>
+  </si>
+  <si>
+    <t>public List&lt;Product&gt; getAllProducts() {
+//        Iterable&lt;Product&gt; it=productRepo.findAll();
+//        ArrayList&lt;Product&gt; products=new ArrayList&lt;&gt;();
+//        it.forEach(products::add);
+//        return products;
+//        return StreamSupport.stream(productRepo.findAll().spliterator(), false)
+//                    .collect(Collectors.toList());
+        return productRepo.findAll();
+    }</t>
+  </si>
+  <si>
+    <t>public List&lt;Product&gt; getAllProducts() {
+        return productRepo.findAll();
+    }</t>
+  </si>
+  <si>
+    <t>Effort to perform tool-based code analysis (hours): 1</t>
   </si>
 </sst>
 </file>
@@ -553,8 +630,30 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -592,28 +691,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -630,6 +709,105 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1495425</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BDF62A12-D8BF-92C4-35A8-242D63CBD52F}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{1162A5B0-8584-104B-FFAF-5164C083838B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3695700" y="1638300"/>
+          <a:ext cx="1495425" cy="676275"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>219075</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{75354AD8-110C-1EF9-71BF-74138A2AF792}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{BDF62A12-D8BF-92C4-35A8-242D63CBD52F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5286375" y="1638300"/>
+          <a:ext cx="1323975" cy="685800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -945,27 +1123,27 @@
       <c r="E1" s="16"/>
       <c r="F1" s="16"/>
       <c r="G1" s="16"/>
-      <c r="H1" s="38" t="s">
+      <c r="H1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="16"/>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
       <c r="F2" s="16"/>
       <c r="G2" s="16"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39" t="s">
+      <c r="H2" s="24"/>
+      <c r="I2" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="39" t="s">
+      <c r="J2" s="24" t="s">
         <v>4</v>
       </c>
     </row>
@@ -977,13 +1155,13 @@
       <c r="E3" s="16"/>
       <c r="F3" s="16"/>
       <c r="G3" s="16"/>
-      <c r="H3" s="39" t="s">
+      <c r="H3" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="39" t="s">
+      <c r="I3" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="39">
+      <c r="J3" s="24">
         <v>237</v>
       </c>
     </row>
@@ -993,44 +1171,54 @@
       <c r="C4" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="19"/>
+      <c r="E4" s="29"/>
       <c r="F4" s="16"/>
       <c r="G4" s="16"/>
-      <c r="H4" s="39" t="s">
+      <c r="H4" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
+      <c r="I4" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="24">
+        <v>237</v>
+      </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="16"/>
       <c r="B5" s="16"/>
       <c r="C5" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="21"/>
+      <c r="D5" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="31"/>
       <c r="F5" s="16"/>
       <c r="G5" s="16"/>
-      <c r="H5" s="39" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="39"/>
-      <c r="J5" s="39"/>
+      <c r="H5" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="24">
+        <v>237</v>
+      </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="16"/>
       <c r="B6" s="7"/>
       <c r="C6" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
+        <v>15</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="26"/>
       <c r="F6" s="16"/>
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
@@ -1041,10 +1229,12 @@
       <c r="A7" s="16"/>
       <c r="B7" s="16"/>
       <c r="C7" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
+        <v>16</v>
+      </c>
+      <c r="D7" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="26"/>
       <c r="F7" s="16"/>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
@@ -1054,16 +1244,16 @@
     <row r="9" spans="1:10">
       <c r="A9" s="16"/>
       <c r="B9" s="9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
@@ -1073,17 +1263,17 @@
     </row>
     <row r="10" spans="1:10" ht="30.75">
       <c r="A10" s="16"/>
-      <c r="B10" s="39">
+      <c r="B10" s="24">
         <v>1</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="30" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F10" s="16"/>
       <c r="G10" s="16"/>
@@ -1093,18 +1283,18 @@
     </row>
     <row r="11" spans="1:10" ht="30.75">
       <c r="A11" s="16"/>
-      <c r="B11" s="39">
+      <c r="B11" s="24">
         <f>B10+1</f>
         <v>2</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
@@ -1114,18 +1304,18 @@
     </row>
     <row r="12" spans="1:10" ht="45.75">
       <c r="A12" s="16"/>
-      <c r="B12" s="39">
+      <c r="B12" s="24">
         <f t="shared" ref="B12:B25" si="0">B11+1</f>
         <v>3</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F12" s="16"/>
       <c r="G12" s="16"/>
@@ -1135,18 +1325,18 @@
     </row>
     <row r="13" spans="1:10" ht="45.75">
       <c r="A13" s="16"/>
-      <c r="B13" s="39">
+      <c r="B13" s="24">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
@@ -1156,16 +1346,16 @@
     </row>
     <row r="14" spans="1:10" ht="45.75">
       <c r="A14" s="16"/>
-      <c r="B14" s="39">
+      <c r="B14" s="24">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
@@ -1175,7 +1365,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="16"/>
-      <c r="B15" s="39">
+      <c r="B15" s="24">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -1190,7 +1380,7 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="16"/>
-      <c r="B16" s="39">
+      <c r="B16" s="24">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
@@ -1204,7 +1394,7 @@
       <c r="J16" s="16"/>
     </row>
     <row r="17" spans="2:5">
-      <c r="B17" s="39">
+      <c r="B17" s="24">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
@@ -1213,81 +1403,81 @@
       <c r="E17" s="2"/>
     </row>
     <row r="18" spans="2:5">
-      <c r="B18" s="39">
+      <c r="B18" s="24">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="40"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="25"/>
     </row>
     <row r="19" spans="2:5">
-      <c r="B19" s="39">
+      <c r="B19" s="24">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="40"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="25"/>
     </row>
     <row r="20" spans="2:5">
-      <c r="B20" s="39">
+      <c r="B20" s="24">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="39"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="40"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="25"/>
     </row>
     <row r="21" spans="2:5">
-      <c r="B21" s="39">
+      <c r="B21" s="24">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="39"/>
-      <c r="D21" s="39"/>
-      <c r="E21" s="40"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="25"/>
     </row>
     <row r="22" spans="2:5">
-      <c r="B22" s="39">
+      <c r="B22" s="24">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="39"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="40"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="25"/>
     </row>
     <row r="23" spans="2:5">
-      <c r="B23" s="39">
+      <c r="B23" s="24">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="39"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="40"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="25"/>
     </row>
     <row r="24" spans="2:5">
-      <c r="B24" s="39">
+      <c r="B24" s="24">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="39"/>
-      <c r="D24" s="39"/>
-      <c r="E24" s="40"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="25"/>
     </row>
     <row r="25" spans="2:5">
-      <c r="B25" s="39">
+      <c r="B25" s="24">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="39"/>
-      <c r="D25" s="39"/>
-      <c r="E25" s="40"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="25"/>
     </row>
     <row r="27" spans="2:5">
       <c r="B27" s="16"/>
       <c r="C27" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D27" s="11"/>
       <c r="E27" s="1">
@@ -1335,27 +1525,27 @@
       <c r="E1" s="16"/>
       <c r="F1" s="16"/>
       <c r="G1" s="16"/>
-      <c r="H1" s="38" t="s">
+      <c r="H1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="16"/>
-      <c r="B2" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
+      <c r="B2" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
       <c r="F2" s="16"/>
       <c r="G2" s="16"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39" t="s">
+      <c r="H2" s="24"/>
+      <c r="I2" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="39" t="s">
+      <c r="J2" s="24" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1367,11 +1557,11 @@
       <c r="E3" s="16"/>
       <c r="F3" s="16"/>
       <c r="G3" s="16"/>
-      <c r="H3" s="39" t="s">
+      <c r="H3" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="39"/>
-      <c r="J3" s="39"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="16"/>
@@ -1379,44 +1569,44 @@
       <c r="C4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" s="22"/>
+      <c r="D4" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="32"/>
       <c r="F4" s="16"/>
       <c r="G4" s="16"/>
-      <c r="H4" s="39" t="s">
+      <c r="H4" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="16"/>
       <c r="B5" s="16"/>
       <c r="C5" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="E5" s="24"/>
+        <v>37</v>
+      </c>
+      <c r="D5" s="33" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="34"/>
       <c r="F5" s="16"/>
       <c r="G5" s="16"/>
-      <c r="H5" s="39" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="39"/>
-      <c r="J5" s="39"/>
+      <c r="H5" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="16"/>
       <c r="B6" s="7"/>
       <c r="C6" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
+        <v>15</v>
+      </c>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
       <c r="F6" s="16"/>
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
@@ -1427,10 +1617,10 @@
       <c r="A7" s="16"/>
       <c r="B7" s="16"/>
       <c r="C7" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
+        <v>16</v>
+      </c>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
       <c r="F7" s="16"/>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
@@ -1440,16 +1630,16 @@
     <row r="9" spans="1:10">
       <c r="A9" s="16"/>
       <c r="B9" s="9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
@@ -1459,17 +1649,17 @@
     </row>
     <row r="10" spans="1:10" ht="43.5">
       <c r="A10" s="16"/>
-      <c r="B10" s="32">
+      <c r="B10" s="18">
         <v>1</v>
       </c>
-      <c r="C10" s="33" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="35" t="s">
-        <v>37</v>
-      </c>
-      <c r="E10" s="35" t="s">
-        <v>38</v>
+      <c r="C10" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>41</v>
       </c>
       <c r="F10" s="16"/>
       <c r="G10" s="16"/>
@@ -1479,17 +1669,17 @@
     </row>
     <row r="11" spans="1:10" ht="43.5">
       <c r="A11" s="16"/>
-      <c r="B11" s="34">
+      <c r="B11" s="20">
         <v>2</v>
       </c>
-      <c r="C11" s="33" t="s">
-        <v>39</v>
-      </c>
-      <c r="D11" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" s="35" t="s">
-        <v>41</v>
+      <c r="C11" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>44</v>
       </c>
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
@@ -1499,17 +1689,17 @@
     </row>
     <row r="12" spans="1:10" ht="83.25">
       <c r="A12" s="16"/>
-      <c r="B12" s="34">
+      <c r="B12" s="20">
         <v>3</v>
       </c>
-      <c r="C12" s="33" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" s="36" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" s="37" t="s">
-        <v>44</v>
+      <c r="C12" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>47</v>
       </c>
       <c r="F12" s="16"/>
       <c r="G12" s="16"/>
@@ -1519,17 +1709,17 @@
     </row>
     <row r="13" spans="1:10" ht="43.5">
       <c r="A13" s="16"/>
-      <c r="B13" s="34">
+      <c r="B13" s="20">
         <v>4</v>
       </c>
-      <c r="C13" s="33" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="E13" s="35" t="s">
-        <v>47</v>
+      <c r="C13" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>50</v>
       </c>
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
@@ -1539,17 +1729,17 @@
     </row>
     <row r="14" spans="1:10" ht="43.5">
       <c r="A14" s="16"/>
-      <c r="B14" s="34">
+      <c r="B14" s="20">
         <v>5</v>
       </c>
-      <c r="C14" s="33" t="s">
-        <v>48</v>
-      </c>
-      <c r="D14" s="35" t="s">
-        <v>49</v>
-      </c>
-      <c r="E14" s="35" t="s">
-        <v>50</v>
+      <c r="C14" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="E14" s="21" t="s">
+        <v>53</v>
       </c>
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
@@ -1559,17 +1749,17 @@
     </row>
     <row r="15" spans="1:10" ht="43.5">
       <c r="A15" s="16"/>
-      <c r="B15" s="34">
+      <c r="B15" s="20">
         <v>6</v>
       </c>
-      <c r="C15" s="33" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" s="35" t="s">
-        <v>52</v>
-      </c>
-      <c r="E15" s="35" t="s">
-        <v>53</v>
+      <c r="C15" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>56</v>
       </c>
       <c r="F15" s="16"/>
       <c r="G15" s="16"/>
@@ -1579,17 +1769,17 @@
     </row>
     <row r="16" spans="1:10" ht="43.5">
       <c r="A16" s="16"/>
-      <c r="B16" s="34">
+      <c r="B16" s="20">
         <v>7</v>
       </c>
-      <c r="C16" s="33" t="s">
-        <v>54</v>
-      </c>
-      <c r="D16" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="E16" s="35" t="s">
-        <v>56</v>
+      <c r="C16" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>59</v>
       </c>
       <c r="F16" s="16"/>
       <c r="G16" s="16"/>
@@ -1598,49 +1788,49 @@
       <c r="J16" s="16"/>
     </row>
     <row r="17" spans="2:5" ht="29.25">
-      <c r="B17" s="34">
+      <c r="B17" s="20">
         <v>8</v>
       </c>
-      <c r="C17" s="33" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" s="35" t="s">
-        <v>37</v>
-      </c>
-      <c r="E17" s="35" t="s">
-        <v>58</v>
+      <c r="C17" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="29.25">
-      <c r="B18" s="34">
+      <c r="B18" s="20">
         <v>9</v>
       </c>
-      <c r="C18" s="33" t="s">
-        <v>59</v>
-      </c>
-      <c r="D18" s="35" t="s">
-        <v>60</v>
-      </c>
-      <c r="E18" s="35" t="s">
-        <v>61</v>
+      <c r="C18" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="D18" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="83.25">
-      <c r="B19" s="34">
+      <c r="B19" s="20">
         <v>10</v>
       </c>
-      <c r="C19" s="33" t="s">
-        <v>62</v>
-      </c>
-      <c r="D19" s="35" t="s">
-        <v>63</v>
-      </c>
-      <c r="E19" s="37" t="s">
-        <v>64</v>
+      <c r="C19" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="D19" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="2:5">
-      <c r="B20" s="39">
+      <c r="B20" s="24">
         <f t="shared" ref="B12:B26" si="0">B19+1</f>
         <v>11</v>
       </c>
@@ -1649,7 +1839,7 @@
       <c r="E20" s="2"/>
     </row>
     <row r="21" spans="2:5">
-      <c r="B21" s="39">
+      <c r="B21" s="24">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
@@ -1658,7 +1848,7 @@
       <c r="E21" s="2"/>
     </row>
     <row r="22" spans="2:5">
-      <c r="B22" s="39">
+      <c r="B22" s="24">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
@@ -1667,7 +1857,7 @@
       <c r="E22" s="2"/>
     </row>
     <row r="23" spans="2:5">
-      <c r="B23" s="39">
+      <c r="B23" s="24">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
@@ -1676,7 +1866,7 @@
       <c r="E23" s="2"/>
     </row>
     <row r="24" spans="2:5">
-      <c r="B24" s="39">
+      <c r="B24" s="24">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
@@ -1685,7 +1875,7 @@
       <c r="E24" s="2"/>
     </row>
     <row r="25" spans="2:5">
-      <c r="B25" s="39">
+      <c r="B25" s="24">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
@@ -1694,7 +1884,7 @@
       <c r="E25" s="2"/>
     </row>
     <row r="26" spans="2:5">
-      <c r="B26" s="39">
+      <c r="B26" s="24">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
@@ -1706,12 +1896,12 @@
       <c r="B27" s="16"/>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
-      <c r="E27" s="31"/>
+      <c r="E27" s="17"/>
     </row>
     <row r="28" spans="2:5">
       <c r="B28" s="16"/>
       <c r="C28" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D28" s="11"/>
       <c r="E28" s="1"/>
@@ -1758,27 +1948,27 @@
       <c r="E1" s="16"/>
       <c r="F1" s="16"/>
       <c r="G1" s="16"/>
-      <c r="H1" s="38" t="s">
+      <c r="H1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="16"/>
-      <c r="B2" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
+      <c r="B2" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
       <c r="F2" s="16"/>
       <c r="G2" s="16"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39" t="s">
+      <c r="H2" s="24"/>
+      <c r="I2" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="39" t="s">
+      <c r="J2" s="24" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1790,11 +1980,11 @@
       <c r="E3" s="16"/>
       <c r="F3" s="16"/>
       <c r="G3" s="16"/>
-      <c r="H3" s="39" t="s">
+      <c r="H3" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="39"/>
-      <c r="J3" s="39"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="16"/>
@@ -1802,44 +1992,44 @@
       <c r="C4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="E4" s="25"/>
+      <c r="D4" s="35" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" s="35"/>
       <c r="F4" s="16"/>
       <c r="G4" s="16"/>
-      <c r="H4" s="39" t="s">
+      <c r="H4" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="16"/>
       <c r="B5" s="16"/>
       <c r="C5" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="E5" s="27"/>
+        <v>11</v>
+      </c>
+      <c r="D5" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="37"/>
       <c r="F5" s="16"/>
       <c r="G5" s="16"/>
-      <c r="H5" s="39" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="39"/>
-      <c r="J5" s="39"/>
+      <c r="H5" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="16"/>
       <c r="B6" s="7"/>
       <c r="C6" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
+        <v>15</v>
+      </c>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
       <c r="F6" s="16"/>
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
@@ -1850,10 +2040,10 @@
       <c r="A7" s="16"/>
       <c r="B7" s="16"/>
       <c r="C7" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
+        <v>16</v>
+      </c>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
       <c r="F7" s="16"/>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
@@ -1863,16 +2053,16 @@
     <row r="9" spans="1:10">
       <c r="A9" s="16"/>
       <c r="B9" s="9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
@@ -1882,7 +2072,7 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="16"/>
-      <c r="B10" s="39">
+      <c r="B10" s="24">
         <v>1</v>
       </c>
       <c r="C10" s="1"/>
@@ -1896,7 +2086,7 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="16"/>
-      <c r="B11" s="39">
+      <c r="B11" s="24">
         <f>B10+1</f>
         <v>2</v>
       </c>
@@ -1911,7 +2101,7 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="16"/>
-      <c r="B12" s="39">
+      <c r="B12" s="24">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
       </c>
@@ -1926,7 +2116,7 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="16"/>
-      <c r="B13" s="39">
+      <c r="B13" s="24">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -1941,7 +2131,7 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="16"/>
-      <c r="B14" s="39">
+      <c r="B14" s="24">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -1956,7 +2146,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="16"/>
-      <c r="B15" s="39">
+      <c r="B15" s="24">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -1971,7 +2161,7 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="16"/>
-      <c r="B16" s="39">
+      <c r="B16" s="24">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
@@ -1985,7 +2175,7 @@
       <c r="J16" s="16"/>
     </row>
     <row r="17" spans="2:5">
-      <c r="B17" s="39">
+      <c r="B17" s="24">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
@@ -1994,7 +2184,7 @@
       <c r="E17" s="2"/>
     </row>
     <row r="18" spans="2:5">
-      <c r="B18" s="39">
+      <c r="B18" s="24">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
@@ -2003,7 +2193,7 @@
       <c r="E18" s="2"/>
     </row>
     <row r="19" spans="2:5">
-      <c r="B19" s="39">
+      <c r="B19" s="24">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -2012,7 +2202,7 @@
       <c r="E19" s="2"/>
     </row>
     <row r="20" spans="2:5">
-      <c r="B20" s="39">
+      <c r="B20" s="24">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
@@ -2021,7 +2211,7 @@
       <c r="E20" s="2"/>
     </row>
     <row r="21" spans="2:5">
-      <c r="B21" s="39">
+      <c r="B21" s="24">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
@@ -2030,7 +2220,7 @@
       <c r="E21" s="2"/>
     </row>
     <row r="22" spans="2:5">
-      <c r="B22" s="39">
+      <c r="B22" s="24">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
@@ -2039,7 +2229,7 @@
       <c r="E22" s="2"/>
     </row>
     <row r="23" spans="2:5">
-      <c r="B23" s="39">
+      <c r="B23" s="24">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
@@ -2048,7 +2238,7 @@
       <c r="E23" s="2"/>
     </row>
     <row r="24" spans="2:5">
-      <c r="B24" s="39">
+      <c r="B24" s="24">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
@@ -2057,7 +2247,7 @@
       <c r="E24" s="2"/>
     </row>
     <row r="25" spans="2:5">
-      <c r="B25" s="39">
+      <c r="B25" s="24">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
@@ -2066,7 +2256,7 @@
       <c r="E25" s="2"/>
     </row>
     <row r="26" spans="2:5">
-      <c r="B26" s="39">
+      <c r="B26" s="24">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
@@ -2075,7 +2265,7 @@
       <c r="E26" s="2"/>
     </row>
     <row r="27" spans="2:5">
-      <c r="B27" s="39">
+      <c r="B27" s="24">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
@@ -2084,7 +2274,7 @@
       <c r="E27" s="1"/>
     </row>
     <row r="28" spans="2:5">
-      <c r="B28" s="39">
+      <c r="B28" s="24">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
@@ -2093,7 +2283,7 @@
       <c r="E28" s="2"/>
     </row>
     <row r="29" spans="2:5">
-      <c r="B29" s="39">
+      <c r="B29" s="24">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
@@ -2102,7 +2292,7 @@
       <c r="E29" s="2"/>
     </row>
     <row r="30" spans="2:5">
-      <c r="B30" s="39">
+      <c r="B30" s="24">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
@@ -2113,7 +2303,7 @@
     <row r="32" spans="2:5">
       <c r="B32" s="16"/>
       <c r="C32" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D32" s="11"/>
       <c r="E32" s="1"/>
@@ -2161,27 +2351,27 @@
       <c r="E1" s="16"/>
       <c r="F1" s="16"/>
       <c r="G1" s="16"/>
-      <c r="H1" s="38" t="s">
+      <c r="H1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="16"/>
-      <c r="B2" s="18" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
+      <c r="B2" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
       <c r="F2" s="16"/>
       <c r="G2" s="16"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39" t="s">
+      <c r="H2" s="24"/>
+      <c r="I2" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="39" t="s">
+      <c r="J2" s="24" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2193,52 +2383,70 @@
       <c r="E3" s="16"/>
       <c r="F3" s="16"/>
       <c r="G3" s="16"/>
-      <c r="H3" s="39" t="s">
+      <c r="H3" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="39"/>
-      <c r="J3" s="39"/>
+      <c r="I3" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="J3" s="24">
+        <v>237</v>
+      </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="16"/>
       <c r="B4" s="16"/>
       <c r="C4" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
+        <v>72</v>
+      </c>
+      <c r="D4" s="35" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" s="35"/>
       <c r="F4" s="16"/>
       <c r="G4" s="16"/>
-      <c r="H4" s="39" t="s">
+      <c r="H4" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
+      <c r="I4" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="24">
+        <v>237</v>
+      </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="16"/>
       <c r="B5" s="16"/>
       <c r="C5" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
+        <v>15</v>
+      </c>
+      <c r="D5" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="26"/>
       <c r="F5" s="16"/>
       <c r="G5" s="16"/>
-      <c r="H5" s="39" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="39"/>
-      <c r="J5" s="39"/>
+      <c r="H5" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="24">
+        <v>237</v>
+      </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="16"/>
       <c r="B6" s="7"/>
       <c r="C6" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
+        <v>16</v>
+      </c>
+      <c r="D6" s="40" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="26"/>
       <c r="F6" s="16"/>
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
@@ -2248,32 +2456,36 @@
     <row r="9" spans="1:10">
       <c r="A9" s="16"/>
       <c r="B9" s="9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
       <c r="J9" s="16"/>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" ht="45.75">
       <c r="A10" s="16"/>
-      <c r="B10" s="39">
+      <c r="B10" s="24">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
+      <c r="C10" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>79</v>
+      </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="16"/>
@@ -2281,61 +2493,91 @@
       <c r="I10" s="16"/>
       <c r="J10" s="16"/>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" ht="91.5">
       <c r="A11" s="16"/>
-      <c r="B11" s="39">
+      <c r="B11" s="24">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>83</v>
+      </c>
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
       <c r="I11" s="16"/>
       <c r="J11" s="16"/>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" ht="137.25">
       <c r="A12" s="16"/>
-      <c r="B12" s="39">
+      <c r="B12" s="24">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>87</v>
+      </c>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
       <c r="J12" s="16"/>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" ht="106.5">
       <c r="A13" s="16"/>
-      <c r="B13" s="39">
+      <c r="B13" s="24">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="C13" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="F13" s="2"/>
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
       <c r="I13" s="16"/>
       <c r="J13" s="16"/>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" ht="305.25">
       <c r="A14" s="16"/>
-      <c r="B14" s="39">
+      <c r="B14" s="24">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
+      <c r="C14" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>93</v>
+      </c>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
@@ -2343,7 +2585,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="16"/>
-      <c r="B15" s="39">
+      <c r="B15" s="24">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -2358,7 +2600,7 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="16"/>
-      <c r="B16" s="39">
+      <c r="B16" s="24">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
@@ -2372,7 +2614,7 @@
       <c r="J16" s="16"/>
     </row>
     <row r="17" spans="2:6">
-      <c r="B17" s="39">
+      <c r="B17" s="24">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
@@ -2382,7 +2624,7 @@
       <c r="F17" s="2"/>
     </row>
     <row r="18" spans="2:6">
-      <c r="B18" s="39">
+      <c r="B18" s="24">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
@@ -2392,7 +2634,7 @@
       <c r="F18" s="2"/>
     </row>
     <row r="19" spans="2:6">
-      <c r="B19" s="39">
+      <c r="B19" s="24">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -2402,7 +2644,7 @@
       <c r="F19" s="2"/>
     </row>
     <row r="20" spans="2:6">
-      <c r="B20" s="39">
+      <c r="B20" s="24">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
@@ -2412,7 +2654,7 @@
       <c r="F20" s="2"/>
     </row>
     <row r="21" spans="2:6">
-      <c r="B21" s="39">
+      <c r="B21" s="24">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
@@ -2422,7 +2664,7 @@
       <c r="F21" s="2"/>
     </row>
     <row r="22" spans="2:6">
-      <c r="B22" s="39">
+      <c r="B22" s="24">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
@@ -2432,7 +2674,7 @@
       <c r="F22" s="2"/>
     </row>
     <row r="23" spans="2:6">
-      <c r="B23" s="39">
+      <c r="B23" s="24">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
@@ -2442,7 +2684,7 @@
       <c r="F23" s="2"/>
     </row>
     <row r="24" spans="2:6">
-      <c r="B24" s="39">
+      <c r="B24" s="24">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
@@ -2452,7 +2694,7 @@
       <c r="F24" s="2"/>
     </row>
     <row r="25" spans="2:6">
-      <c r="B25" s="39">
+      <c r="B25" s="24">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
@@ -2462,7 +2704,7 @@
       <c r="F25" s="2"/>
     </row>
     <row r="26" spans="2:6">
-      <c r="B26" s="39">
+      <c r="B26" s="24">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
@@ -2472,7 +2714,7 @@
       <c r="F26" s="2"/>
     </row>
     <row r="27" spans="2:6">
-      <c r="B27" s="39">
+      <c r="B27" s="24">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
@@ -2482,7 +2724,7 @@
       <c r="F27" s="1"/>
     </row>
     <row r="28" spans="2:6">
-      <c r="B28" s="39">
+      <c r="B28" s="24">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
@@ -2492,7 +2734,7 @@
       <c r="F28" s="2"/>
     </row>
     <row r="29" spans="2:6">
-      <c r="B29" s="39">
+      <c r="B29" s="24">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
@@ -2502,7 +2744,7 @@
       <c r="F29" s="2"/>
     </row>
     <row r="30" spans="2:6">
-      <c r="B30" s="39">
+      <c r="B30" s="24">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
@@ -2513,11 +2755,11 @@
     </row>
     <row r="32" spans="2:6">
       <c r="B32" s="16"/>
-      <c r="C32" s="28" t="s">
-        <v>74</v>
-      </c>
-      <c r="D32" s="29"/>
-      <c r="E32" s="29"/>
+      <c r="C32" s="38" t="s">
+        <v>94</v>
+      </c>
+      <c r="D32" s="39"/>
+      <c r="E32" s="39"/>
       <c r="F32" s="15"/>
     </row>
     <row r="35" spans="6:6">
@@ -2534,5 +2776,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>